<commit_message>
update full w19 y 18
</commit_message>
<xml_diff>
--- a/checkrates/week-20/Analisis_Checkrates_B2C_7d.xlsx
+++ b/checkrates/week-20/Analisis_Checkrates_B2C_7d.xlsx
@@ -541,7 +541,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 03:55 · W20 · 12-18 may 2026</t>
+          <t>Generado: 19/05/2026 04:09 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 03:55 · W20 · 12-18 may 2026</t>
+          <t>Generado: 19/05/2026 04:09 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 03:55 · W20 · 12-18 may 2026</t>
+          <t>Generado: 19/05/2026 04:09 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 03:55 · W20 · 12-18 may 2026</t>
+          <t>Generado: 19/05/2026 04:09 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -6247,7 +6247,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 03:55 · W20 · 12-18 may 2026</t>
+          <t>Generado: 19/05/2026 04:09 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -10546,7 +10546,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 03:55 · W20 · 12-18 may 2026</t>
+          <t>Generado: 19/05/2026 04:09 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12844,7 +12844,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 03:55 · W20 · 12-18 may 2026</t>
+          <t>Generado: 19/05/2026 04:09 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16438,7 +16438,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 03:55 · W20 · 12-18 may 2026</t>
+          <t>Generado: 19/05/2026 04:09 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16777,7 +16777,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 03:55 · W20 · 12-18 may 2026</t>
+          <t>Generado: 19/05/2026 04:09 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>